<commit_message>
fix: atualiza cache do mapa por timestamp e inclui bases no bat
</commit_message>
<xml_diff>
--- a/data/bases_hubs.xlsx
+++ b/data/bases_hubs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\opera\Desktop\app\bases_hubs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\opera\Desktop\app\dashboard_operacao\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF27C9B-404E-409F-843E-06C56EC76760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EB5D51-D58A-4520-9765-BFFAAC2193EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0855A8E1-0FF3-4F9E-B54B-0B4ED6505555}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Planilha2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$H$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$H$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="297">
   <si>
     <t>ID</t>
   </si>
@@ -705,9 +705,6 @@
     <t>PAIM</t>
   </si>
   <si>
-    <t>MATRIZ</t>
-  </si>
-  <si>
     <t>MAYLES</t>
   </si>
   <si>
@@ -729,9 +726,6 @@
     <t>TMB_GOV_VALADARES</t>
   </si>
   <si>
-    <t>TMB_VIANA</t>
-  </si>
-  <si>
     <t>TMB_UBERLANDIA</t>
   </si>
   <si>
@@ -874,6 +868,72 @@
   </si>
   <si>
     <t>Palmas</t>
+  </si>
+  <si>
+    <t>LOGCARE_MATRIZ</t>
+  </si>
+  <si>
+    <t>06612-000</t>
+  </si>
+  <si>
+    <t>Via de Acesso João de Góes,2300</t>
+  </si>
+  <si>
+    <t>Jardim Alvorada</t>
+  </si>
+  <si>
+    <t>Jandira</t>
+  </si>
+  <si>
+    <t>PORTO VELHO</t>
+  </si>
+  <si>
+    <t>RO</t>
+  </si>
+  <si>
+    <t>76816-880</t>
+  </si>
+  <si>
+    <t>Rua Sevilha,QD 16 LT 204</t>
+  </si>
+  <si>
+    <t>Aeroclube</t>
+  </si>
+  <si>
+    <t>Porto Velho</t>
+  </si>
+  <si>
+    <t>TMB_VITÓRIA</t>
+  </si>
+  <si>
+    <t>MARABÁ</t>
+  </si>
+  <si>
+    <t>68507-445</t>
+  </si>
+  <si>
+    <t>Quadra Quinze,LT 17</t>
+  </si>
+  <si>
+    <t>Nova Marabá</t>
+  </si>
+  <si>
+    <t>Marabá</t>
+  </si>
+  <si>
+    <t>DOURADOS</t>
+  </si>
+  <si>
+    <t>79896-000</t>
+  </si>
+  <si>
+    <t>R Barão do Rio Branco,225</t>
+  </si>
+  <si>
+    <t>Itapora</t>
+  </si>
+  <si>
+    <t>Mato Grosso do Sul</t>
   </si>
 </sst>
 </file>
@@ -1334,7 +1394,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9291FB8C-A7CD-482C-9F46-A943A8F45085}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
@@ -1379,22 +1439,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>220</v>
+        <v>275</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>276</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>8</v>
+        <v>277</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>9</v>
+        <v>278</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>10</v>
+        <v>279</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>86</v>
@@ -1457,7 +1517,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>21</v>
@@ -1483,7 +1543,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>26</v>
@@ -1509,7 +1569,7 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>31</v>
@@ -1535,7 +1595,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>36</v>
@@ -1743,7 +1803,7 @@
         <v>21</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
@@ -1873,22 +1933,22 @@
         <v>28</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="E21" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>248</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>86</v>
@@ -1899,22 +1959,22 @@
         <v>29</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>194</v>
       </c>
       <c r="D22" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>253</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>86</v>
@@ -1925,22 +1985,22 @@
         <v>30</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>11</v>
       </c>
       <c r="D23" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>256</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>86</v>
@@ -1951,22 +2011,22 @@
         <v>31</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="E24" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>262</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>86</v>
@@ -1977,22 +2037,22 @@
         <v>32</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="E25" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>268</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>270</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>86</v>
@@ -2003,22 +2063,22 @@
         <v>33</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="E26" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>274</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>276</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>86</v>
@@ -2029,25 +2089,25 @@
         <v>34</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>224</v>
+        <v>280</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>46</v>
+        <v>281</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>202</v>
+        <v>282</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>103</v>
+        <v>283</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>120</v>
+        <v>284</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>87</v>
+        <v>285</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -2055,22 +2115,22 @@
         <v>35</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>225</v>
+        <v>286</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>46</v>
+        <v>102</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>85</v>
@@ -2078,25 +2138,25 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>85</v>
@@ -2104,77 +2164,77 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>227</v>
+        <v>287</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>46</v>
+        <v>194</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>205</v>
+        <v>288</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>106</v>
+        <v>289</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>122</v>
+        <v>290</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>84</v>
+        <v>291</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>38</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>228</v>
+        <v>39</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>292</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>102</v>
+        <v>264</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>90</v>
+        <v>293</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>296</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>85</v>
@@ -2182,51 +2242,51 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="2">
-        <v>41</v>
+      <c r="A34" s="1">
+        <v>42</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>85</v>
@@ -2234,25 +2294,25 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>85</v>
@@ -2260,51 +2320,51 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="2">
-        <v>44</v>
+      <c r="A37" s="1">
+        <v>45</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>85</v>
@@ -2312,25 +2372,25 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>85</v>
@@ -2338,51 +2398,51 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="2">
-        <v>47</v>
+      <c r="A40" s="1">
+        <v>48</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>85</v>
@@ -2390,25 +2450,25 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>85</v>
@@ -2416,53 +2476,131 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="2">
-        <v>50</v>
+      <c r="A43" s="1">
+        <v>51</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C43" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" s="2">
+        <v>52</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D44" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="2">
+        <v>53</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>54</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E46" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F46" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G43" s="3" t="s">
+      <c r="G46" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>